<commit_message>
Add Remark column for NOT_FOUND accounts based on screenshot analysis
</commit_message>
<xml_diff>
--- a/dspm_consolidated_status.xlsx
+++ b/dspm_consolidated_status.xlsx
@@ -14,10 +14,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ERROR" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'COMPLETED'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RUNNING'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'NOT_FOUND'!$A$1:$P$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ERROR'!$A$1:$P$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'COMPLETED'!$A$1:$Q$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'RUNNING'!$A$1:$Q$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'NOT_FOUND'!$A$1:$Q$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'ERROR'!$A$1:$Q$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -772,7 +772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:Q23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -791,6 +791,7 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="33" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -874,6 +875,11 @@
           <t>Screenshot File</t>
         </is>
       </c>
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
@@ -956,6 +962,7 @@
           <t>odl_user_2226954_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q2" s="9" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -1034,6 +1041,7 @@
           <t>odl_user_2226956_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q3" s="9" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
@@ -1112,6 +1120,7 @@
           <t>odl_user_2226957_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q4" s="9" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
@@ -1190,6 +1199,7 @@
           <t>odl_user_2226963_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q5" s="9" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
@@ -1272,6 +1282,7 @@
           <t>odl_user_2226964_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q6" s="9" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
@@ -1354,6 +1365,7 @@
           <t>odl_user_2226972_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q7" s="9" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
@@ -1432,6 +1444,7 @@
           <t>odl_user_2226991_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q8" s="9" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
@@ -1510,6 +1523,7 @@
           <t>odl_user_2227014_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q9" s="9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
@@ -1588,6 +1602,7 @@
           <t>odl_user_2227016_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q10" s="9" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
@@ -1670,6 +1685,7 @@
           <t>odl_user_2227017_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q11" s="9" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
@@ -1748,6 +1764,7 @@
           <t>odl_user_2227034_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q12" s="9" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
@@ -1826,6 +1843,7 @@
         </is>
       </c>
       <c r="P13" s="9" t="inlineStr"/>
+      <c r="Q13" s="9" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
@@ -1900,6 +1918,7 @@
         </is>
       </c>
       <c r="P14" s="9" t="inlineStr"/>
+      <c r="Q14" s="9" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
@@ -1978,6 +1997,7 @@
           <t>odl_user_2227049_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q15" s="9" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
@@ -2056,6 +2076,7 @@
           <t>odl_user_2227050_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q16" s="9" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -2134,6 +2155,7 @@
           <t>odl_user_2227051_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q17" s="9" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
@@ -2212,6 +2234,7 @@
           <t>odl_user_2227052_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q18" s="9" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
@@ -2290,6 +2313,7 @@
           <t>odl_user_2227066_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q19" s="9" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
@@ -2372,6 +2396,7 @@
           <t>odl_user_2227067_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q20" s="9" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
@@ -2450,6 +2475,7 @@
           <t>odl_user_2227097_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q21" s="9" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
@@ -2528,6 +2554,7 @@
           <t>odl_user_2227115_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q22" s="9" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
@@ -2606,9 +2633,10 @@
           <t>odl_user_2227114_COMPLETED.png</t>
         </is>
       </c>
+      <c r="Q23" s="9" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P1"/>
+  <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2619,7 +2647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P180"/>
+  <dimension ref="A1:Q180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2638,6 +2666,7 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="31" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2721,6 +2750,11 @@
           <t>Screenshot File</t>
         </is>
       </c>
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="10" t="inlineStr">
@@ -2791,6 +2825,7 @@
           <t>odl_user_2227227_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q2" s="10" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="10" t="inlineStr">
@@ -2861,6 +2896,7 @@
           <t>odl_user_2227228_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q3" s="10" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="10" t="inlineStr">
@@ -2931,6 +2967,7 @@
           <t>odl_user_2226966_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q4" s="10" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
@@ -3001,6 +3038,7 @@
           <t>odl_user_2227229_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q5" s="10" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="10" t="inlineStr">
@@ -3071,6 +3109,7 @@
           <t>odl_user_2226967_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q6" s="10" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
@@ -3141,6 +3180,7 @@
           <t>odl_user_2226971_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q7" s="10" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="10" t="inlineStr">
@@ -3211,6 +3251,7 @@
           <t>odl_user_2226969_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q8" s="10" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
@@ -3281,6 +3322,7 @@
           <t>odl_user_2227230_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q9" s="10" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="10" t="inlineStr">
@@ -3351,6 +3393,7 @@
           <t>odl_user_2226979_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q10" s="10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
@@ -3421,6 +3464,7 @@
           <t>odl_user_2227231_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q11" s="10" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="10" t="inlineStr">
@@ -3491,6 +3535,7 @@
           <t>odl_user_2226975_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q12" s="10" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
@@ -3561,6 +3606,7 @@
           <t>odl_user_2226978_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q13" s="10" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="10" t="inlineStr">
@@ -3631,6 +3677,7 @@
           <t>odl_user_2226977_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q14" s="10" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
@@ -3701,6 +3748,7 @@
           <t>odl_user_2226980_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q15" s="10" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="inlineStr">
@@ -3771,6 +3819,7 @@
           <t>odl_user_2226981_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q16" s="10" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
@@ -3841,6 +3890,7 @@
           <t>odl_user_2226985_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q17" s="10" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="10" t="inlineStr">
@@ -3911,6 +3961,7 @@
           <t>odl_user_2226982_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q18" s="10" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
@@ -3981,6 +4032,7 @@
           <t>odl_user_2226986_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q19" s="10" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="10" t="inlineStr">
@@ -4051,6 +4103,7 @@
           <t>odl_user_2226990_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q20" s="10" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="10" t="inlineStr">
@@ -4121,6 +4174,7 @@
           <t>odl_user_2227004_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q21" s="10" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
@@ -4191,6 +4245,7 @@
           <t>odl_user_2226995_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q22" s="10" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
@@ -4261,6 +4316,7 @@
           <t>odl_user_2226994_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q23" s="10" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="10" t="inlineStr">
@@ -4331,6 +4387,7 @@
           <t>odl_user_2227005_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q24" s="10" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="10" t="inlineStr">
@@ -4401,6 +4458,7 @@
           <t>odl_user_2227008_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q25" s="10" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
@@ -4471,6 +4529,7 @@
           <t>odl_user_2227007_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q26" s="10" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
@@ -4541,6 +4600,7 @@
           <t>odl_user_2227010_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q27" s="10" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="10" t="inlineStr">
@@ -4611,6 +4671,7 @@
           <t>odl_user_2227232_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q28" s="10" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
@@ -4679,6 +4740,7 @@
           <t>odl_user_2227018_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q29" s="10" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="10" t="inlineStr">
@@ -4749,6 +4811,7 @@
           <t>odl_user_2227019_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q30" s="10" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
@@ -4819,6 +4882,7 @@
           <t>odl_user_2227020_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q31" s="10" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="10" t="inlineStr">
@@ -4889,6 +4953,7 @@
           <t>odl_user_2227022_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q32" s="10" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="10" t="inlineStr">
@@ -4959,6 +5024,7 @@
           <t>odl_user_2227024_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q33" s="10" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="10" t="inlineStr">
@@ -5029,6 +5095,7 @@
           <t>odl_user_2227025_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q34" s="10" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="10" t="inlineStr">
@@ -5099,6 +5166,7 @@
           <t>odl_user_2227029_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q35" s="10" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="10" t="inlineStr">
@@ -5169,6 +5237,7 @@
           <t>odl_user_2227031_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q36" s="10" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="inlineStr">
@@ -5239,6 +5308,7 @@
           <t>odl_user_2227030_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q37" s="10" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="10" t="inlineStr">
@@ -5309,6 +5379,7 @@
           <t>odl_user_2227032_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q38" s="10" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="10" t="inlineStr">
@@ -5379,6 +5450,7 @@
           <t>odl_user_2227033_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q39" s="10" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="10" t="inlineStr">
@@ -5449,6 +5521,7 @@
           <t>odl_user_2227035_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q40" s="10" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="10" t="inlineStr">
@@ -5519,6 +5592,7 @@
           <t>odl_user_2227036_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q41" s="10" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="10" t="inlineStr">
@@ -5589,6 +5663,7 @@
           <t>odl_user_2227234_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q42" s="10" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="10" t="inlineStr">
@@ -5659,6 +5734,7 @@
           <t>odl_user_2227235_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q43" s="10" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="10" t="inlineStr">
@@ -5729,6 +5805,7 @@
           <t>odl_user_2227038_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q44" s="10" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="inlineStr">
@@ -5799,6 +5876,7 @@
           <t>odl_user_2227037_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q45" s="10" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="10" t="inlineStr">
@@ -5869,6 +5947,7 @@
           <t>odl_user_2227236_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q46" s="10" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="10" t="inlineStr">
@@ -5939,6 +6018,7 @@
           <t>odl_user_2227040_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q47" s="10" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="10" t="inlineStr">
@@ -6009,6 +6089,7 @@
           <t>odl_user_2227237_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q48" s="10" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="10" t="inlineStr">
@@ -6079,6 +6160,7 @@
           <t>odl_user_2227238_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q49" s="10" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="10" t="inlineStr">
@@ -6149,6 +6231,7 @@
           <t>odl_user_2227240_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q50" s="10" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="10" t="inlineStr">
@@ -6219,6 +6302,7 @@
           <t>odl_user_2227045_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q51" s="10" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
@@ -6289,6 +6373,7 @@
           <t>odl_user_2227044_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q52" s="10" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
@@ -6359,6 +6444,7 @@
           <t>odl_user_2227042_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q53" s="10" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="10" t="inlineStr">
@@ -6429,6 +6515,7 @@
           <t>odl_user_2227046_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q54" s="10" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
@@ -6499,6 +6586,7 @@
           <t>odl_user_2227047_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q55" s="10" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="10" t="inlineStr">
@@ -6569,6 +6657,7 @@
           <t>odl_user_2227053_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q56" s="10" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
@@ -6639,6 +6728,7 @@
           <t>odl_user_2227241_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q57" s="10" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="10" t="inlineStr">
@@ -6709,6 +6799,7 @@
           <t>odl_user_2227054_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q58" s="10" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
@@ -6779,6 +6870,7 @@
           <t>odl_user_2227055_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q59" s="10" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="inlineStr">
@@ -6849,6 +6941,7 @@
           <t>odl_user_2227057_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q60" s="10" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
@@ -6919,6 +7012,7 @@
           <t>odl_user_2227056_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q61" s="10" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
@@ -6989,6 +7083,7 @@
           <t>odl_user_2227243_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q62" s="10" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
@@ -7057,6 +7152,7 @@
           <t>odl_user_2227060_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q63" s="10" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="10" t="inlineStr">
@@ -7127,6 +7223,7 @@
           <t>odl_user_2227061_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q64" s="10" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
@@ -7193,6 +7290,7 @@
           <t>odl_user_2227063_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q65" s="10" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="10" t="inlineStr">
@@ -7263,6 +7361,7 @@
           <t>odl_user_2227065_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q66" s="10" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
@@ -7333,6 +7432,7 @@
           <t>odl_user_2227070_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q67" s="10" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="10" t="inlineStr">
@@ -7403,6 +7503,7 @@
           <t>odl_user_2227068_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q68" s="10" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
@@ -7473,6 +7574,7 @@
           <t>odl_user_2227244_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q69" s="10" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="10" t="inlineStr">
@@ -7543,6 +7645,7 @@
           <t>odl_user_2227072_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q70" s="10" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
@@ -7613,6 +7716,7 @@
           <t>odl_user_2227071_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q71" s="10" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="10" t="inlineStr">
@@ -7683,6 +7787,7 @@
           <t>odl_user_2227075_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q72" s="10" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
@@ -7753,6 +7858,7 @@
           <t>odl_user_2227074_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q73" s="10" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="10" t="inlineStr">
@@ -7823,6 +7929,7 @@
           <t>odl_user_2227076_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q74" s="10" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
@@ -7893,6 +8000,7 @@
           <t>odl_user_2227077_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q75" s="10" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="10" t="inlineStr">
@@ -7963,6 +8071,7 @@
           <t>odl_user_2227078_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q76" s="10" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
@@ -8033,6 +8142,7 @@
           <t>odl_user_2227079_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q77" s="10" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="10" t="inlineStr">
@@ -8103,6 +8213,7 @@
           <t>odl_user_2227080_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q78" s="10" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
@@ -8173,6 +8284,7 @@
           <t>odl_user_2227081_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q79" s="10" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="10" t="inlineStr">
@@ -8243,6 +8355,7 @@
           <t>odl_user_2227083_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q80" s="10" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
@@ -8313,6 +8426,7 @@
           <t>odl_user_2227084_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q81" s="10" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="10" t="inlineStr">
@@ -8383,6 +8497,7 @@
           <t>odl_user_2227245_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q82" s="10" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
@@ -8453,6 +8568,7 @@
           <t>odl_user_2227086_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q83" s="10" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="10" t="inlineStr">
@@ -8523,6 +8639,7 @@
           <t>odl_user_2227088_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q84" s="10" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
@@ -8593,6 +8710,7 @@
           <t>odl_user_2227085_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q85" s="10" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="10" t="inlineStr">
@@ -8663,6 +8781,7 @@
           <t>odl_user_2227087_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q86" s="10" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
@@ -8733,6 +8852,7 @@
           <t>odl_user_2227089_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q87" s="10" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="10" t="inlineStr">
@@ -8803,6 +8923,7 @@
           <t>odl_user_2227246_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q88" s="10" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
@@ -8873,6 +8994,7 @@
           <t>odl_user_2227090_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q89" s="10" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="10" t="inlineStr">
@@ -8943,6 +9065,7 @@
           <t>odl_user_2227082_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q90" s="10" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
@@ -9013,6 +9136,7 @@
           <t>odl_user_2227095_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q91" s="10" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="10" t="inlineStr">
@@ -9083,6 +9207,7 @@
           <t>odl_user_2227092_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q92" s="10" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
@@ -9153,6 +9278,7 @@
           <t>odl_user_2227094_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q93" s="10" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="10" t="inlineStr">
@@ -9223,6 +9349,7 @@
           <t>odl_user_2227096_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q94" s="10" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
@@ -9293,6 +9420,7 @@
           <t>odl_user_2227098_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q95" s="10" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="10" t="inlineStr">
@@ -9363,6 +9491,7 @@
           <t>odl_user_2227099_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q96" s="10" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
@@ -9433,6 +9562,7 @@
           <t>odl_user_2227100_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q97" s="10" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="10" t="inlineStr">
@@ -9503,6 +9633,7 @@
           <t>odl_user_2227101_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q98" s="10" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
@@ -9573,6 +9704,7 @@
           <t>odl_user_2227102_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q99" s="10" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="10" t="inlineStr">
@@ -9643,6 +9775,7 @@
           <t>odl_user_2227103_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q100" s="10" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
@@ -9713,6 +9846,7 @@
           <t>odl_user_2227104_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q101" s="10" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="10" t="inlineStr">
@@ -9783,6 +9917,7 @@
           <t>odl_user_2227105_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q102" s="10" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
@@ -9853,6 +9988,7 @@
           <t>odl_user_2227106_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q103" s="10" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="10" t="inlineStr">
@@ -9923,6 +10059,7 @@
           <t>odl_user_2227107_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q104" s="10" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
@@ -9993,6 +10130,7 @@
           <t>odl_user_2227108_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q105" s="10" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="10" t="inlineStr">
@@ -10063,6 +10201,7 @@
           <t>odl_user_2227109_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q106" s="10" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
@@ -10133,6 +10272,7 @@
           <t>odl_user_2227111_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q107" s="10" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="10" t="inlineStr">
@@ -10203,6 +10343,7 @@
           <t>odl_user_2227112_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q108" s="10" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
@@ -10273,6 +10414,7 @@
           <t>odl_user_2227110_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q109" s="10" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="10" t="inlineStr">
@@ -10343,6 +10485,7 @@
           <t>odl_user_2227113_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q110" s="10" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
@@ -10413,6 +10556,7 @@
           <t>odl_user_2227116_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q111" s="10" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="10" t="inlineStr">
@@ -10483,6 +10627,7 @@
           <t>odl_user_2227117_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q112" s="10" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
@@ -10553,6 +10698,7 @@
           <t>odl_user_2227118_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q113" s="10" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="10" t="inlineStr">
@@ -10623,6 +10769,7 @@
           <t>odl_user_2227120_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q114" s="10" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
@@ -10693,6 +10840,7 @@
           <t>odl_user_2227119_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q115" s="10" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="10" t="inlineStr">
@@ -10763,6 +10911,7 @@
           <t>odl_user_2227125_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q116" s="10" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
@@ -10833,6 +10982,7 @@
           <t>odl_user_2227121_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q117" s="10" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="10" t="inlineStr">
@@ -10903,6 +11053,7 @@
           <t>odl_user_2227123_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q118" s="10" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
@@ -10971,6 +11122,7 @@
           <t>odl_user_2227127_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q119" s="10" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="10" t="inlineStr">
@@ -11041,6 +11193,7 @@
           <t>odl_user_2227128_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q120" s="10" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
@@ -11111,6 +11264,7 @@
           <t>odl_user_2227130_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q121" s="10" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="10" t="inlineStr">
@@ -11181,6 +11335,7 @@
           <t>odl_user_2227132_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q122" s="10" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
@@ -11251,6 +11406,7 @@
           <t>odl_user_2227133_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q123" s="10" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="10" t="inlineStr">
@@ -11321,6 +11477,7 @@
           <t>odl_user_2227134_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q124" s="10" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
@@ -11391,6 +11548,7 @@
           <t>odl_user_2227135_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q125" s="10" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" s="10" t="inlineStr">
@@ -11461,6 +11619,7 @@
           <t>odl_user_2227136_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q126" s="10" t="inlineStr"/>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
@@ -11531,6 +11690,7 @@
           <t>odl_user_2227139_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q127" s="10" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="10" t="inlineStr">
@@ -11601,6 +11761,7 @@
           <t>odl_user_2227141_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q128" s="10" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
@@ -11671,6 +11832,7 @@
           <t>odl_user_2227144_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q129" s="10" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="10" t="inlineStr">
@@ -11741,6 +11903,7 @@
           <t>odl_user_2227145_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q130" s="10" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
@@ -11811,6 +11974,7 @@
           <t>odl_user_2227143_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q131" s="10" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="10" t="inlineStr">
@@ -11881,6 +12045,7 @@
           <t>odl_user_2227146_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q132" s="10" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
@@ -11951,6 +12116,7 @@
           <t>odl_user_2227148_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q133" s="10" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="10" t="inlineStr">
@@ -12021,6 +12187,7 @@
           <t>odl_user_2227150_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q134" s="10" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
@@ -12091,6 +12258,7 @@
           <t>odl_user_2227149_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q135" s="10" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="10" t="inlineStr">
@@ -12161,6 +12329,7 @@
           <t>odl_user_2227147_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q136" s="10" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
@@ -12231,6 +12400,7 @@
           <t>odl_user_2227152_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q137" s="10" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="10" t="inlineStr">
@@ -12301,6 +12471,7 @@
           <t>odl_user_2227153_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q138" s="10" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="10" t="inlineStr">
@@ -12371,6 +12542,7 @@
           <t>odl_user_2227155_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q139" s="10" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" s="10" t="inlineStr">
@@ -12441,6 +12613,7 @@
           <t>odl_user_2227156_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q140" s="10" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="10" t="inlineStr">
@@ -12511,6 +12684,7 @@
           <t>odl_user_2227158_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q141" s="10" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="10" t="inlineStr">
@@ -12577,6 +12751,7 @@
           <t>odl_user_2227157_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q142" s="10" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="10" t="inlineStr">
@@ -12647,6 +12822,7 @@
           <t>odl_user_2227159_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q143" s="10" t="inlineStr"/>
     </row>
     <row r="144">
       <c r="A144" s="10" t="inlineStr">
@@ -12717,6 +12893,7 @@
           <t>odl_user_2227160_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q144" s="10" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="10" t="inlineStr">
@@ -12785,6 +12962,7 @@
           <t>odl_user_2227162_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q145" s="10" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="10" t="inlineStr">
@@ -12855,6 +13033,7 @@
           <t>odl_user_2227163_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q146" s="10" t="inlineStr"/>
     </row>
     <row r="147">
       <c r="A147" s="10" t="inlineStr">
@@ -12925,6 +13104,7 @@
           <t>odl_user_2227164_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q147" s="10" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" s="10" t="inlineStr">
@@ -12995,6 +13175,7 @@
           <t>odl_user_2227165_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q148" s="10" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" s="10" t="inlineStr">
@@ -13065,6 +13246,7 @@
           <t>odl_user_2227166_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q149" s="10" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="10" t="inlineStr">
@@ -13135,6 +13317,7 @@
           <t>odl_user_2227167_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q150" s="10" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="10" t="inlineStr">
@@ -13205,6 +13388,7 @@
           <t>odl_user_2227169_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q151" s="10" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="10" t="inlineStr">
@@ -13275,6 +13459,7 @@
           <t>odl_user_2227170_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q152" s="10" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="10" t="inlineStr">
@@ -13345,6 +13530,7 @@
           <t>odl_user_2227171_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q153" s="10" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="10" t="inlineStr">
@@ -13415,6 +13601,7 @@
           <t>odl_user_2227173_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q154" s="10" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="10" t="inlineStr">
@@ -13485,6 +13672,7 @@
           <t>odl_user_2227172_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q155" s="10" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" s="10" t="inlineStr">
@@ -13555,6 +13743,7 @@
           <t>odl_user_2227174_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q156" s="10" t="inlineStr"/>
     </row>
     <row r="157">
       <c r="A157" s="10" t="inlineStr">
@@ -13625,6 +13814,7 @@
           <t>odl_user_2227175_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q157" s="10" t="inlineStr"/>
     </row>
     <row r="158">
       <c r="A158" s="10" t="inlineStr">
@@ -13695,6 +13885,7 @@
           <t>odl_user_2227177_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q158" s="10" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" s="10" t="inlineStr">
@@ -13765,6 +13956,7 @@
           <t>odl_user_2227176_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q159" s="10" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" s="10" t="inlineStr">
@@ -13835,6 +14027,7 @@
           <t>odl_user_2227179_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q160" s="10" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="10" t="inlineStr">
@@ -13905,6 +14098,7 @@
           <t>odl_user_2227180_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q161" s="10" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" s="10" t="inlineStr">
@@ -13975,6 +14169,7 @@
           <t>odl_user_2227253_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q162" s="10" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" s="10" t="inlineStr">
@@ -14045,6 +14240,7 @@
           <t>odl_user_2227182_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q163" s="10" t="inlineStr"/>
     </row>
     <row r="164">
       <c r="A164" s="10" t="inlineStr">
@@ -14115,6 +14311,7 @@
           <t>odl_user_2227183_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q164" s="10" t="inlineStr"/>
     </row>
     <row r="165">
       <c r="A165" s="10" t="inlineStr">
@@ -14185,6 +14382,7 @@
           <t>odl_user_2227184_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q165" s="10" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" s="10" t="inlineStr">
@@ -14255,6 +14453,7 @@
           <t>odl_user_2227185_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q166" s="10" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" s="10" t="inlineStr">
@@ -14325,6 +14524,7 @@
           <t>odl_user_2227187_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q167" s="10" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" s="10" t="inlineStr">
@@ -14395,6 +14595,7 @@
           <t>odl_user_2227186_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q168" s="10" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" s="10" t="inlineStr">
@@ -14465,6 +14666,7 @@
           <t>odl_user_2227188_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q169" s="10" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" s="10" t="inlineStr">
@@ -14535,6 +14737,7 @@
           <t>odl_user_2227190_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q170" s="10" t="inlineStr"/>
     </row>
     <row r="171">
       <c r="A171" s="10" t="inlineStr">
@@ -14605,6 +14808,7 @@
           <t>odl_user_2227191_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q171" s="10" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" s="10" t="inlineStr">
@@ -14675,6 +14879,7 @@
           <t>odl_user_2227192_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q172" s="10" t="inlineStr"/>
     </row>
     <row r="173">
       <c r="A173" s="10" t="inlineStr">
@@ -14745,6 +14950,7 @@
           <t>odl_user_2227193_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q173" s="10" t="inlineStr"/>
     </row>
     <row r="174">
       <c r="A174" s="10" t="inlineStr">
@@ -14815,6 +15021,7 @@
           <t>odl_user_2227197_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q174" s="10" t="inlineStr"/>
     </row>
     <row r="175">
       <c r="A175" s="10" t="inlineStr">
@@ -14885,6 +15092,7 @@
           <t>odl_user_2227194_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q175" s="10" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" s="10" t="inlineStr">
@@ -14955,6 +15163,7 @@
           <t>odl_user_2227198_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q176" s="10" t="inlineStr"/>
     </row>
     <row r="177">
       <c r="A177" s="10" t="inlineStr">
@@ -15025,6 +15234,7 @@
           <t>odl_user_2227200_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q177" s="10" t="inlineStr"/>
     </row>
     <row r="178">
       <c r="A178" s="10" t="inlineStr">
@@ -15095,6 +15305,7 @@
           <t>odl_user_2227201_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q178" s="10" t="inlineStr"/>
     </row>
     <row r="179">
       <c r="A179" s="10" t="inlineStr">
@@ -15165,6 +15376,7 @@
           <t>odl_user_2227199_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q179" s="10" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" s="10" t="inlineStr">
@@ -15235,9 +15447,10 @@
           <t>odl_user_2227202_RUNNING.png</t>
         </is>
       </c>
+      <c r="Q180" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P1"/>
+  <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -15248,7 +15461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P67"/>
+  <dimension ref="A1:Q67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -15267,6 +15480,7 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="33" customWidth="1" min="16" max="16"/>
+    <col width="53" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -15350,6 +15564,11 @@
           <t>Screenshot File</t>
         </is>
       </c>
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
@@ -15420,6 +15639,11 @@
           <t>odl_user_2226984_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q2" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
@@ -15490,6 +15714,11 @@
           <t>odl_user_2226992_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q3" s="11" t="inlineStr">
+        <is>
+          <t>Switch to classic portal dialog blocking content</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="11" t="inlineStr">
@@ -15556,6 +15785,11 @@
           <t>odl_user_2227842_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q4" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -15622,6 +15856,11 @@
           <t>odl_user_2227843_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q5" s="11" t="inlineStr">
+        <is>
+          <t>Switch to classic portal dialog blocking content</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="11" t="inlineStr">
@@ -15692,6 +15931,11 @@
           <t>odl_user_2227021_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q6" s="11" t="inlineStr">
+        <is>
+          <t>Switch to classic portal dialog blocking content</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="11" t="inlineStr">
@@ -15762,6 +16006,11 @@
           <t>odl_user_2227233_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q7" s="11" t="inlineStr">
+        <is>
+          <t>Switch to classic portal dialog blocking content</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="11" t="inlineStr">
@@ -15832,6 +16081,11 @@
           <t>odl_user_2227039_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q8" s="11" t="inlineStr">
+        <is>
+          <t>Login failed - stuck on Microsoft Sign-in page</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
@@ -15902,6 +16156,11 @@
           <t>odl_user_2227043_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q9" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="11" t="inlineStr">
@@ -15972,6 +16231,11 @@
           <t>odl_user_2227242_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q10" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -16042,6 +16306,11 @@
           <t>odl_user_2227059_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q11" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="11" t="inlineStr">
@@ -16108,6 +16377,11 @@
           <t>odl_user_2227844_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q12" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
@@ -16174,6 +16448,11 @@
           <t>odl_user_2227845_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q13" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="11" t="inlineStr">
@@ -16244,6 +16523,11 @@
           <t>odl_user_2227091_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q14" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Asset explorer page</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
@@ -16314,6 +16598,11 @@
           <t>odl_user_2227093_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q15" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Asset explorer page</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="inlineStr">
@@ -16384,6 +16673,11 @@
           <t>odl_user_2227131_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q16" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Asset explorer page</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
@@ -16454,6 +16748,11 @@
           <t>odl_user_2227126_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q17" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Asset explorer page</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="11" t="inlineStr">
@@ -16524,6 +16823,11 @@
           <t>odl_user_2227129_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q18" s="11" t="inlineStr">
+        <is>
+          <t>Page loading timeout - spinner/shimmer visible</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="11" t="inlineStr">
@@ -16590,6 +16894,11 @@
           <t>odl_user_2227855_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q19" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Asset explorer page</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="11" t="inlineStr">
@@ -16656,6 +16965,11 @@
           <t>odl_user_2227848_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q20" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Asset explorer page</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="11" t="inlineStr">
@@ -16722,6 +17036,11 @@
           <t>odl_user_2227856_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q21" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
@@ -16792,6 +17111,11 @@
           <t>odl_user_2227168_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q22" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Asset explorer page</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="11" t="inlineStr">
@@ -16862,6 +17186,11 @@
           <t>odl_user_2227178_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q23" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Asset explorer page</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
@@ -16928,6 +17257,11 @@
           <t>odl_user_2227846_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q24" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -16998,6 +17332,11 @@
           <t>odl_user_2227196_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q25" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
@@ -17068,6 +17407,11 @@
           <t>odl_user_2227195_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q26" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="11" t="inlineStr">
@@ -17134,6 +17478,11 @@
           <t>odl_user_2227511_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q27" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
@@ -17200,6 +17549,11 @@
           <t>odl_user_2227510_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q28" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="11" t="inlineStr">
@@ -17266,6 +17620,11 @@
           <t>odl_user_2227512_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q29" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="11" t="inlineStr">
@@ -17332,6 +17691,11 @@
           <t>odl_user_2227513_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q30" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="11" t="inlineStr">
@@ -17398,6 +17762,11 @@
           <t>odl_user_2227414_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q31" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="11" t="inlineStr">
@@ -17464,6 +17833,11 @@
           <t>odl_user_2227418_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q32" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="11" t="inlineStr">
@@ -17530,6 +17904,11 @@
           <t>odl_user_2227421_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q33" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="11" t="inlineStr">
@@ -17596,6 +17975,11 @@
           <t>odl_user_2227423_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q34" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="11" t="inlineStr">
@@ -17662,6 +18046,11 @@
           <t>odl_user_2227821_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q35" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="11" t="inlineStr">
@@ -17728,6 +18117,11 @@
           <t>odl_user_2227827_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q36" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
@@ -17794,6 +18188,11 @@
           <t>odl_user_2227812_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q37" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
@@ -17860,6 +18259,11 @@
           <t>odl_user_2227813_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q38" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
@@ -17926,6 +18330,11 @@
           <t>odl_user_2227496_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q39" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
@@ -17992,6 +18401,11 @@
           <t>odl_user_2227498_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q40" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="11" t="inlineStr">
@@ -18058,6 +18472,11 @@
           <t>odl_user_2227495_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q41" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="11" t="inlineStr">
@@ -18124,6 +18543,11 @@
           <t>odl_user_2227500_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q42" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="11" t="inlineStr">
@@ -18190,6 +18614,11 @@
           <t>odl_user_2227501_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q43" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
@@ -18256,6 +18685,11 @@
           <t>odl_user_2227502_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q44" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
@@ -18322,6 +18756,11 @@
           <t>odl_user_2227503_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q45" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="11" t="inlineStr">
@@ -18388,6 +18827,11 @@
           <t>odl_user_2227506_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q46" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="11" t="inlineStr">
@@ -18454,6 +18898,11 @@
           <t>odl_user_2227507_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q47" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="11" t="inlineStr">
@@ -18520,6 +18969,11 @@
           <t>odl_user_2227825_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q48" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="11" t="inlineStr">
@@ -18586,6 +19040,11 @@
           <t>odl_user_2227508_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q49" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="11" t="inlineStr">
@@ -18644,6 +19103,11 @@
           <t>odl_user_2227331_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q50" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="11" t="inlineStr">
@@ -18702,6 +19166,11 @@
           <t>odl_user_2227342_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q51" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="11" t="inlineStr">
@@ -18760,6 +19229,11 @@
           <t>odl_user_2227322_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q52" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="11" t="inlineStr">
@@ -18818,6 +19292,11 @@
           <t>odl_user_2227321_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q53" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="11" t="inlineStr">
@@ -18876,6 +19355,11 @@
           <t>odl_user_2227324_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q54" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="11" t="inlineStr">
@@ -18934,6 +19418,11 @@
           <t>odl_user_2227323_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q55" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="11" t="inlineStr">
@@ -18992,6 +19481,11 @@
           <t>odl_user_2227325_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q56" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="11" t="inlineStr">
@@ -19050,6 +19544,11 @@
           <t>odl_user_2227332_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q57" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="11" t="inlineStr">
@@ -19108,6 +19607,11 @@
           <t>odl_user_2227345_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q58" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="11" t="inlineStr">
@@ -19166,6 +19670,11 @@
           <t>odl_user_2227343_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q59" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="11" t="inlineStr">
@@ -19224,6 +19733,11 @@
           <t>odl_user_2227335_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q60" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="11" t="inlineStr">
@@ -19282,6 +19796,11 @@
           <t>odl_user_2227330_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q61" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="11" t="inlineStr">
@@ -19340,6 +19859,11 @@
           <t>odl_user_2227326_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q62" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="11" t="inlineStr">
@@ -19398,6 +19922,11 @@
           <t>odl_user_2227337_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q63" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="11" t="inlineStr">
@@ -19456,6 +19985,11 @@
           <t>odl_user_2227327_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q64" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="11" t="inlineStr">
@@ -19514,6 +20048,11 @@
           <t>odl_user_2227346_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q65" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="11" t="inlineStr">
@@ -19572,6 +20111,11 @@
           <t>odl_user_2227339_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q66" s="11" t="inlineStr">
+        <is>
+          <t>Insufficient permissions - needs Purview Content Analyst role</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="11" t="inlineStr">
@@ -19630,9 +20174,14 @@
           <t>odl_user_2227328_NOT_FOUND.png</t>
         </is>
       </c>
+      <c r="Q67" s="11" t="inlineStr">
+        <is>
+          <t>Blank/empty Posture Agent tab</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P1"/>
+  <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -19643,7 +20192,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -19662,6 +20211,7 @@
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="22" customWidth="1" min="15" max="15"/>
     <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -19745,6 +20295,11 @@
           <t>Screenshot File</t>
         </is>
       </c>
+      <c r="Q1" s="8" t="inlineStr">
+        <is>
+          <t>Remark</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
@@ -19799,9 +20354,10 @@
         </is>
       </c>
       <c r="P2" s="12" t="inlineStr"/>
+      <c r="Q2" s="12" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P1"/>
+  <autoFilter ref="A1:Q1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>